<commit_message>
Add how_to_redeem_short field to all Gyftr brands
Short 1-2 line redemption summaries generated for each of the 380
brands in data/gyftr_master.json (mirrored into db/gyftr_master.json
and gyftr_full_database.xlsx), following: online-vs-offline step
condensing based on redemption_type, no URLs/login instructions,
plain Indian English. 18 brands with missing/blank redemption data
got null instead of a guessed summary.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gyftr_full_database.xlsx
+++ b/gyftr_full_database.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S381"/>
+  <dimension ref="A1:T381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -550,6 +550,11 @@
           <t>Last Scraped</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>How to Redeem (Short)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -625,6 +630,11 @@
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -709,6 +719,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Under AJIO Wallet, tap 'Have a Gift Card?' → 'Add' → enter your voucher code and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -788,6 +803,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -865,6 +885,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>At cart, click 'Apply Offers and Coupons' → enter your Gift Voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -942,6 +967,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1021,6 +1051,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1096,6 +1131,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>At checkout, apply your gift card under 'Apply Coupon Code'.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1173,6 +1213,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1252,6 +1297,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>At checkout, select 'GyFTR e-Pay' → enter your voucher code to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1331,6 +1381,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>In your Air India Wallet, enter your gift card number and PIN, then tap Add.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1414,6 +1469,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>In your Air India Wallet, enter your gift card number and PIN, then tap Add.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1497,6 +1557,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>In your Air India Wallet, enter your gift card number and PIN, then tap Add.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1570,6 +1635,11 @@
       <c r="S14" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>At payment, tap 'Add Promo Code' → enter your code and pay Rs.1 to activate.</t>
         </is>
       </c>
     </row>
@@ -1652,6 +1722,11 @@
       <c r="S15" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Under AJIO Wallet, tap 'Have a Gift Card?' → 'Add' → enter your voucher code and PIN.</t>
         </is>
       </c>
     </row>
@@ -1733,6 +1808,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>After selecting your plan, enter your voucher code and redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1811,6 +1891,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Under 'Amazon Pay - Add Gift Card', enter your gift card code to add it to your Amazon Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1888,6 +1973,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Under 'Claim New', enter your voucher code and click 'Add to your Vouchers'.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1969,6 +2059,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Under 'Add to Your Vouchers', enter your 13-digit voucher code to activate Prime.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2050,6 +2145,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Under 'Add New', enter your Shopping Voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2125,6 +2225,11 @@
       <c r="S21" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -2205,6 +2310,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>In the app, go to 'All Coupons &amp; Vouchers' → select Gift Voucher → enter code + PIN → tap 'Use Voucher'.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2284,6 +2394,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Tap 'Redeem Gift Card or Code' and enter your voucher number manually.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2361,6 +2476,11 @@
       <c r="S24" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -2443,6 +2563,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Add product to cart → tap 'Add' and enter voucher code to top up your balance.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2520,6 +2645,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2599,6 +2729,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2674,6 +2809,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2751,6 +2891,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code under 'Discount' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2828,6 +2973,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay with GyFTR' → enter your voucher details.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2903,6 +3053,11 @@
       <c r="S31" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -2985,6 +3140,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>In the Hello BPCL app, add your Fuel Voucher under 'Add a Corporate Gift Voucher' to recharge, then authenticate with OTP at the pump.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3062,6 +3222,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Voucher code under 'Enter Coupon Code' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3139,6 +3304,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3220,6 +3390,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3293,6 +3468,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3372,6 +3548,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3451,6 +3632,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3530,6 +3716,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3607,6 +3798,11 @@
       <c r="S40" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -3689,6 +3885,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3768,6 +3969,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3845,6 +4051,11 @@
       <c r="S43" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>At checkout, select 'E-pay' → verify with OTP → add your voucher to your ePay balance.</t>
         </is>
       </c>
     </row>
@@ -3928,6 +4139,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Tap the top-right icon → 'My Gift Cards' → enter voucher number + PIN to credit your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4008,6 +4224,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4085,6 +4306,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4162,6 +4388,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Enter your voucher code in the field provided, then choose a subscription plan to redeem against it.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4239,6 +4470,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4318,6 +4554,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4395,6 +4636,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4474,6 +4720,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>At checkout, enter your e-Pay/GV code and click Add → enter the amount and click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4553,6 +4804,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4630,6 +4886,11 @@
       <c r="S53" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -4710,6 +4971,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → enter your voucher code to add to your ePay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4789,6 +5055,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4864,6 +5135,11 @@
       <c r="S56" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -4944,6 +5220,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>At payment, check 'Pay with GYFTR' → enter your voucher number and captcha, then Submit.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5020,6 +5301,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>At payment, check 'Pay with GYFTR' → enter your voucher number and captcha, then Submit.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5098,6 +5384,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>At payment, check 'Pay with GYFTR' → enter your voucher number and captcha, then Submit.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5175,6 +5466,11 @@
       <c r="S60" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>At checkout, choose 'Pay via e-Pay/Gift Vouchers' and enter your voucher code.</t>
         </is>
       </c>
     </row>
@@ -5250,6 +5546,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Apply your Gift Card at payment and pay any remaining amount by card or cash.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5329,6 +5630,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number or voucher code with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5408,6 +5714,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher under 'Gift Voucher - ePay' and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5485,6 +5796,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>At payment, click 'Apply Coupon' → enter your voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5568,6 +5884,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Before payment, enter your 16-digit gift card number and PIN under 'Apply Coupon or Gift Card'.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5651,6 +5972,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Before payment, enter your 16-digit gift card number and PIN under 'Apply Coupon or Gift Card'.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5726,6 +6052,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher in the 'Apply Coupon' section.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5801,6 +6132,11 @@
       <c r="S68" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -5883,6 +6219,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5962,6 +6303,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6041,6 +6387,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>At checkout, select 'GyFTR Gift Card' → verify with OTP → enter the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6116,6 +6467,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6193,6 +6545,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Card Voucher' → enter voucher number and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6270,6 +6627,11 @@
       <c r="S74" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>At checkout, choose 'Gyftr ePay' → apply your voucher and enter the amount to redeem.</t>
         </is>
       </c>
     </row>
@@ -6351,6 +6713,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>In the app, go to 'Redeem Gift Card' → enter your unique code.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6429,6 +6796,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>In the Domino's app cart, choose 'Gift Card / e-Voucher' and enter your voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6506,6 +6878,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>At payment, choose the 'E-Gift Card' option to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6585,6 +6962,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6662,6 +7044,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Under 'Redeem Gift Card', enter your voucher ID and PIN, then click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6741,6 +7128,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>At payment, select 'Have a Gift Card' → enter voucher code + PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6818,6 +7210,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6893,6 +7290,11 @@
       <c r="S82" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>On the Buy Plan page, click 'Apply Voucher' → enter your voucher code.</t>
         </is>
       </c>
     </row>
@@ -6966,6 +7368,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7047,6 +7450,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7124,6 +7528,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7199,6 +7608,11 @@
       <c r="S86" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -7281,6 +7695,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>At payment, choose 'Gift Card' → enter your card number and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7356,6 +7775,11 @@
       <c r="S88" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Tell the cashier you want to use a Gift Card and share the card details with them.</t>
         </is>
       </c>
     </row>
@@ -7438,6 +7862,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7512,6 +7941,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>On the payment summary, click 'Apply Coupon/Gift Card' → enter your code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7593,6 +8027,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7672,6 +8107,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code under 'Discount Coupon' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7749,6 +8189,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7826,6 +8271,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7903,6 +8353,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Card code(s) -- up to 5 per order.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7980,6 +8435,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Voucher code and click 'Redeem Now' (or 'Apply GyFTR Coupon').</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8057,6 +8517,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Voucher code and click 'Redeem Now' (or 'Apply GyFTR Coupon').</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8134,6 +8599,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8211,6 +8681,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>In the app, select 'GyFTR Voucher' → verify with OTP → add the voucher to your FITCASH balance.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -8288,6 +8763,11 @@
       <c r="S100" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Gift Card' → enter your voucher code and the amount to redeem.</t>
         </is>
       </c>
     </row>
@@ -8370,6 +8850,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay with GyFTR' → enter the amount you want to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8450,6 +8935,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8527,6 +9017,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>While booking, select 'Have a gift voucher code?' → enter voucher code and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8604,6 +9099,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8685,6 +9185,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8762,6 +9263,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8837,6 +9343,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8914,6 +9421,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8991,6 +9503,11 @@
       <c r="S109" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
         </is>
       </c>
     </row>
@@ -9072,6 +9589,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>On the cart page, click 'Have a Discount Coupon' → enter voucher code and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -9154,6 +9676,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Under 'Saved Cards &amp; Wallets', tap 'Add Flipkart Gift Card' → enter voucher code + PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -9231,6 +9758,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>At payment, select 'Enter Coupon' and enter your voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -9308,6 +9840,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>At payment summary, click 'Have a Coupon Code?' → enter your voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -9387,6 +9924,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>At checkout, add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9464,6 +10006,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>At cart, enter your 10-digit gift card code under 'Enter Coupon Code'.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9543,6 +10090,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>At checkout, select the ePay option to pay with your Gift Card.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9620,6 +10172,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9701,6 +10258,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9781,6 +10339,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>In the app, tap 'Redeem GIVA ePay' → verify with OTP → enter the amount to redeem and tap Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9861,6 +10424,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>In the app, tap 'Redeem GIVA ePay' → verify with OTP → enter the amount to redeem and tap Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9937,6 +10505,11 @@
       <c r="S121" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -10018,6 +10591,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Under Settings → Subscriptions, tap 'Redeem Coupon' → enter your code and proceed.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10099,6 +10677,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -10174,6 +10753,11 @@
       <c r="S124" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -10233,6 +10817,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10312,6 +10897,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>At checkout, select 'e-Pay' → enter your GV code and the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -10387,6 +10977,11 @@
       <c r="S127" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -10468,6 +11063,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>In the HP Pay app, tap 'Add Voucher' to top up your wallet, then scan and pay at the pump.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -10545,6 +11145,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10622,6 +11227,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code under 'Coupon Code' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10701,6 +11311,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>At checkout, select the ePay option to pay with your Gift Card.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10776,6 +11391,11 @@
       <c r="S132" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>Under account → 'HK Cash', enter your Gift Card number under 'Avail HK Cash through Gift Card'.</t>
         </is>
       </c>
     </row>
@@ -10858,6 +11478,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>At checkout, redeem your GyFTR E-Gift Card → verify with OTP → enter the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10931,6 +11556,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>Under 'Activate Plan', enter your unique coupon code.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -11006,6 +11636,11 @@
       <c r="S135" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -11086,6 +11721,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Gift Voucher e-pay' → enter voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -11163,6 +11803,11 @@
       <c r="S137" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -11243,6 +11888,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>After choosing your plan, enter your coupon code and click 'Apply Coupon'.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -11320,6 +11970,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>Under 'Redeem Code', enter your subscription code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -11397,6 +12052,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -11474,6 +12134,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -11551,6 +12216,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -11628,6 +12298,11 @@
       <c r="S143" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -11703,6 +12378,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code in the details form before payment.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -11781,6 +12461,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Under Profile → Wallet, enter your voucher code and apply to top up your wallet balance.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -11856,6 +12541,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Under 'My Vouchers', select 'Claim Voucher' → enter your code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11929,6 +12619,11 @@
       <c r="S147" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Share your voucher code and registered mobile number at the POS machine.</t>
         </is>
       </c>
     </row>
@@ -12011,6 +12706,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Under Auto Pay, select 'Gift Voucher' → 'GyFTR' → enter your mobile number to view and add vouchers → redeem with OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -12088,6 +12788,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>At check-out, share your 16-digit card number and the OTP sent to your registered mobile number.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12167,6 +12872,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Gift Card' option to apply your voucher.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12246,6 +12956,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -12325,6 +13040,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>At checkout, select the ePay option to pay with your Gift Card.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -12402,6 +13122,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>In Offers, tap 'Have a Coupon Code?' → enter your voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -12479,6 +13204,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -12556,6 +13286,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>After OTP login, enter your voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12631,6 +13366,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -12708,6 +13444,11 @@
       <c r="S157" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>Under profile, tap 'Jockey Credit' → 'Add Gift Card' → enter voucher number and captcha, then Apply.</t>
         </is>
       </c>
     </row>
@@ -12790,6 +13531,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Add Balance to GyFTR E-Pay' → enter your voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -12863,6 +13609,11 @@
       <c r="S159" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>At payment, choose 'Gift Card' → enter voucher code + PIN.</t>
         </is>
       </c>
     </row>
@@ -12938,6 +13689,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -13011,6 +13767,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -13082,6 +13843,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13160,6 +13926,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>At checkout, choose the 'Gyftr' option to pay via Gift Card.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -13235,6 +14006,11 @@
       <c r="S164" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -13315,6 +14091,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>At checkout, click 'Pay Online' → enter your voucher number under 'Voucher Number' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -13393,6 +14174,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher number in the 'Voucher Number' field and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -13471,6 +14257,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher number in the 'Voucher Number' field and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -13550,6 +14341,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>At checkout, click 'Use ePay Voucher' → enter your code and select 'Add Gift Voucher to ePay'.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -13625,6 +14421,11 @@
       <c r="S169" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>Under Accounts → 'Promo Codes', enter your voucher and click Redeem.</t>
         </is>
       </c>
     </row>
@@ -13707,6 +14508,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>Under 'My Profile', tap 'Claim Gift Card' → enter your code + PIN and click Claim.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -13784,6 +14590,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -13865,6 +14676,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -13945,6 +14757,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>At checkout, choose 'Pay via e-pay/Gift Vouchers' → enter your voucher details and the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -14024,6 +14841,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -14103,6 +14925,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher under 'Gift Voucher - ePay' and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -14180,6 +15007,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -14257,6 +15089,11 @@
       <c r="S177" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>At checkout, click 'Have a Gift Card' → enter your 16-digit card number and PIN.</t>
         </is>
       </c>
     </row>
@@ -14337,6 +15174,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>Choose 'Voucher' as payment method → enter your voucher code and click Continue.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -14414,6 +15256,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>Click 'Have a Coupon' → enter your code and click 'Apply Coupon'.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -14491,6 +15338,11 @@
       <c r="S180" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>At payment, choose 'Gyftr Wallet' → verify with OTP → add your voucher and apply the e-Pay balance.</t>
         </is>
       </c>
     </row>
@@ -14573,6 +15425,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -14650,6 +15507,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -14727,6 +15589,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -14804,6 +15671,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -14887,6 +15759,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>Under 'Redeem', enter your voucher code in the 'Redeem Your Code or Gift Card' section.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -14962,6 +15839,11 @@
       <c r="S186" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -15037,6 +15919,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -15114,6 +16001,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -15191,6 +16083,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>At payment, tap 'Gift Cards' → 'Add MMT e-Pay Gift Card' → enter your 16-digit code and verify with OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -15268,6 +16165,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>At payment, tap 'Gift Cards' → 'Add MMT e-Pay Gift Card' → enter your 16-digit code and verify with OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -15343,6 +16245,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>At payment, tap 'Gift Cards' → 'Add MMT e-Pay Gift Card' → enter your 16-digit code and verify with OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -15420,6 +16327,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>At payment, under 'Gift Cards', click Apply → enter card number + PIN → Add and Confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -15497,6 +16409,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>At payment, under 'Gift Cards', click Apply → enter card number + PIN → Add and Confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -15574,6 +16491,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>At payment, under 'Gift Cards', click Apply → enter card number + PIN → Add and Confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -15647,6 +16569,11 @@
       <c r="S195" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>At payment, under 'Gift Card' option, enter your card details and click Apply.</t>
         </is>
       </c>
     </row>
@@ -15725,6 +16652,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>At checkout, add your voucher to your E-Pay balance or enter the code manually.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -15804,6 +16736,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -15881,6 +16818,11 @@
       <c r="S198" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -15962,6 +16904,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>At checkout, select 'GyFTR EPAY' → verify with OTP → add your voucher and redeem the amount.</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -16039,6 +16986,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code and apply it.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -16118,6 +17070,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>At checkout, click 'Have a Gift Card' → enter your 16-digit card number and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -16197,6 +17154,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher under 'Gift Voucher - ePay' and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -16274,6 +17236,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>At payment, choose 'Gift Voucher' and enter your voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -16351,6 +17318,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -16428,6 +17400,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -16511,6 +17488,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>Under 'Redeem', enter your voucher code in the 'Redeem Your Code or Gift Card' section.</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -16590,6 +17572,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>Under 'Redeem', enter your voucher code in the 'Redeem Your Code or Gift Card' section.</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -16669,6 +17656,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>In your wallet, choose the 'GV/e-Pay' option → add and redeem your voucher.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -16748,6 +17740,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>At checkout, select 'GyFTR ePay' → enter your voucher code under Recharge to add balance.</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -16829,6 +17826,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -16910,6 +17908,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -16987,6 +17986,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -17060,6 +18064,11 @@
       <c r="S213" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>At checkout, add your gift voucher manually to redeem.</t>
         </is>
       </c>
     </row>
@@ -17146,6 +18155,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>Under Payment &amp; Currencies, tap 'Myntra Credit' → 'Add Gift Card' → enter voucher code + PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -17225,6 +18239,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -17304,6 +18323,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>At checkout, select the Gift Voucher option to pay with your Gift Card.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -17383,6 +18407,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -17462,6 +18491,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher under 'Gift Voucher - ePay' and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -17541,6 +18575,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -17620,6 +18659,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>At checkout, choose the 'GyFTR voucher/e-Pay' option to view and add your vouchers.</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -17701,6 +18745,11 @@
       <c r="S221" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>At checkout, select 'GyFTR E-Pay' → enter your voucher and click Add.</t>
         </is>
       </c>
     </row>
@@ -17788,6 +18837,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Card' → enter your 16-digit code + PIN and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -17873,6 +18927,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Card' → enter your 16-digit code + PIN and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -17958,6 +19017,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Card' → enter your 16-digit code + PIN and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -18036,6 +19100,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>In the app, tap 'Apply Coupon' → enter your voucher code and apply.</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -18115,6 +19184,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -18190,6 +19264,11 @@
       <c r="S227" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
         </is>
       </c>
     </row>
@@ -18272,6 +19351,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -18345,6 +19429,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -18422,6 +19507,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -18499,6 +19589,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -18576,6 +19671,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -18653,6 +19753,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -18728,6 +19833,11 @@
       <c r="S234" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -18813,6 +19923,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>While booking, click the 'GyFTR' option → enter your Gift Voucher number.</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -18890,6 +20005,11 @@
       <c r="S236" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code and click Apply, then select your e-Pay balance to apply it.</t>
         </is>
       </c>
     </row>
@@ -18972,6 +20092,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -19052,6 +20177,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -19131,6 +20261,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>At checkout, enter your GyFTR e-Pay/GV code to add it, then enter the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -19210,6 +20345,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>Share your voucher code and mobile number with the cashier, then confirm with the OTP you receive.</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -19285,6 +20425,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -19358,6 +20499,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -19435,6 +20581,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>Under Donor options, select Redeem → 'Gyftr Voucher' → enter your voucher code, then choose your charity.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -19512,6 +20663,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>Under 'Coupons &amp; Offers', enter your voucher code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -19589,6 +20745,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -19668,6 +20829,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>At checkout, log in via mobile number to access your Gift Card balance → enter the amount to redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -19743,6 +20909,11 @@
       <c r="S247" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -19825,6 +20996,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>In the app, go to Pronto Money → 'Claim a Gift Card' → enter your voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -19900,6 +21076,11 @@
       <c r="S249" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -19982,6 +21163,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -20056,6 +21242,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>Enter your Gift Voucher code (without hyphens) as the Product Key during setup or activation.</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -20135,6 +21326,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -20212,6 +21408,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -20289,6 +21490,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -20366,6 +21572,11 @@
       <c r="S255" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay with GyFTR' → enter your voucher details.</t>
         </is>
       </c>
     </row>
@@ -20448,6 +21659,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -20521,6 +21737,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code and click 'Apply Now'.</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -20600,6 +21821,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -20675,6 +21901,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -20748,6 +21979,11 @@
       <c r="S260" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -20828,6 +22064,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Add Gift Card/Voucher Code' → enter your 16-digit code and redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -20905,6 +22146,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -20980,6 +22226,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -21057,6 +22308,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -21132,6 +22388,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -21209,6 +22470,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -21284,6 +22550,11 @@
       <c r="S267" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -21359,6 +22630,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code and proceed to payment.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -21432,6 +22708,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>Click the Robux icon → 'Redeem Roblox Codes' → enter your voucher and click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -21509,6 +22790,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>Click the Robux icon → 'Redeem Roblox Codes' → enter your voucher and click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -21586,6 +22872,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -21665,6 +22956,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -21744,6 +23040,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -21819,6 +23120,11 @@
       <c r="S274" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -21894,6 +23200,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code and select your payment option.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -21971,6 +23282,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T276" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -22048,6 +23364,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -22125,6 +23446,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -22200,6 +23526,11 @@
       <c r="S279" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -22277,6 +23608,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>Click 'Check Offers/Coupons' → enter your voucher number and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -22352,6 +23688,11 @@
       <c r="S281" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>Under Profile → 'Redeem Code', enter your 10-digit code and click Apply.</t>
         </is>
       </c>
     </row>
@@ -22431,6 +23772,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Voucher or discount code.</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -22508,6 +23854,11 @@
       <c r="S283" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Card code under 'Use Coupons' and click Apply.</t>
         </is>
       </c>
     </row>
@@ -22590,6 +23941,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>At cart, select 'E-Gift Voucher' → enter voucher number, PIN and amount, then click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -22667,6 +24023,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>At checkout, click 'Have a promo code?' → enter your code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -22746,6 +24107,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher under 'Apply Vouchers' → click Apply → confirm with your mobile number.</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -22823,6 +24189,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -22902,6 +24273,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>At payment, select 'GyFTR' → place order and verify with OTP → tap 'Add Voucher' to apply.</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -22977,6 +24353,11 @@
       <c r="S289" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>Select 'Redeem Voucher' → choose GyFTR as partner → verify with OTP → add your coupon.</t>
         </is>
       </c>
     </row>
@@ -23059,6 +24440,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>At payment, select 'GyFTR e-Pay Balance' → add your voucher code and click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -23132,6 +24518,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>Under your profile, select 'Redeem Code' → enter your 12-digit voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -23209,6 +24600,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Under 'Do you have a coupon', enter your code and click 'Activate Offer'.</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -23288,6 +24684,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>At checkout, tap 'Add' under 'Add Balance to Your ePay' → enter your voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -23365,6 +24766,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Gift Card/Gift Voucher' → enter your voucher number and captcha.</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -23446,6 +24852,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -23517,6 +24924,11 @@
       <c r="S296" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>Under 'Enter Your Premium Code', enter your voucher code and continue.</t>
         </is>
       </c>
     </row>
@@ -23600,6 +25012,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>In the Starbucks app, add your card under 'Starbucks Pay' → show the barcode to the cashier to scan.</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -23675,6 +25092,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>Under Wallet → 'Add Funds' → 'Redeem a Steam Gift Card' → enter your code.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -23754,6 +25176,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>Under Wallet → 'Add Funds' → 'Redeem a Steam Gift Card' → enter your code.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -23831,6 +25258,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -23910,6 +25342,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
@@ -23987,6 +25424,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -24064,6 +25506,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>At checkout, enter your gift card details in the 'Gift Card' box.</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -24141,6 +25588,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -24220,6 +25672,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T305" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gyftr - Epay' → tap Pay Now and enter your gift card.</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
@@ -24295,6 +25752,11 @@
       <c r="S306" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T306" t="inlineStr">
+        <is>
+          <t>Inform the cashier about your Gift Voucher before ordering, then show the code again at billing.</t>
         </is>
       </c>
     </row>
@@ -24377,6 +25839,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -24452,6 +25919,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>At checkout, tap 'Apply Coupon Code' → enter your voucher and redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -24531,6 +26003,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>Under Account → 'Swiggy Money', tap 'Add Voucher' → enter your voucher code and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -24612,6 +26089,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T310" t="inlineStr">
+        <is>
+          <t>Under Account → 'Swiggy Money', tap 'Add Voucher' → enter your voucher code and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
@@ -24685,6 +26167,11 @@
       <c r="S311" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T311" t="inlineStr">
+        <is>
+          <t>Under 'One Membership', tap 'Redeem 3rd Party Coupon' → enter your voucher code.</t>
         </is>
       </c>
     </row>
@@ -24768,6 +26255,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T312" t="inlineStr">
+        <is>
+          <t>Under CLiQ Cash, enter your gift card code to add balance → apply CLiQ Cash at payment.</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
@@ -24849,6 +26341,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>At checkout, enter your Gift Voucher code under 'Gift Card or Discount Code'.</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -24926,6 +26423,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
@@ -25003,6 +26505,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T315" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -25080,6 +26587,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T316" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
@@ -25157,6 +26669,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T317" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number or voucher code with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
@@ -25234,6 +26751,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T318" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -25313,6 +26835,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T319" t="inlineStr">
+        <is>
+          <t>Share your card number and PIN at the reception when booking or checking in.</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -25390,6 +26917,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T320" t="inlineStr">
+        <is>
+          <t>Present your voucher at the spa reception before payment.</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -25469,6 +27001,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>Share your 16-digit voucher code and 6-digit validation code with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -25544,6 +27081,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T322" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -25621,6 +27163,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T323" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
@@ -25698,6 +27245,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T324" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -25773,6 +27325,11 @@
       <c r="S325" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T325" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -25856,6 +27413,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T326" t="inlineStr">
+        <is>
+          <t>Under CLiQ Cash, enter your gift card code to add balance → apply CLiQ Cash at payment.</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -25933,6 +27495,11 @@
       <c r="S327" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T327" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay with GyFTR' to redeem your voucher.</t>
         </is>
       </c>
     </row>
@@ -26013,6 +27580,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T328" t="inlineStr">
+        <is>
+          <t>At checkout, enter your voucher code under 'Apply Gift Card' → verify with OTP → pay using 'Pay from wallet'.</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -26093,6 +27665,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T329" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -26170,6 +27747,11 @@
       <c r="S330" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T330" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
         </is>
       </c>
     </row>
@@ -26250,6 +27832,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T331" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -26325,6 +27912,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T332" t="inlineStr">
+        <is>
+          <t>At cart, enter your unique discount code and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -26402,6 +27994,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T333" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -26481,6 +28078,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T334" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -26556,6 +28158,11 @@
       <c r="S335" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T335" t="inlineStr">
+        <is>
+          <t>Show your Gift Voucher at the cash counter before billing.</t>
         </is>
       </c>
     </row>
@@ -26636,6 +28243,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T336" t="inlineStr">
+        <is>
+          <t>Under Account Settings → 'Promo Code', enter your voucher code and click Submit.</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -26713,6 +28325,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T337" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -26790,6 +28407,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T338" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -26867,6 +28489,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T339" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
@@ -26942,6 +28569,11 @@
       <c r="S340" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T340" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -27017,6 +28649,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T341" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Voucher' option and enter your voucher code.</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
@@ -27096,6 +28733,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T342" t="inlineStr">
+        <is>
+          <t>In Order Summary, tap 'ePay Balance' → 'Add Balance' → enter your voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -27173,6 +28815,11 @@
       <c r="S343" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T343" t="inlineStr">
+        <is>
+          <t>In the app, go to Account → Wallet → '+Add voucher code' → enter your code and confirm.</t>
         </is>
       </c>
     </row>
@@ -27254,6 +28901,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T344" t="inlineStr">
+        <is>
+          <t>Tap '+' to add a voucher → select 'UniPin Physical Voucher' → enter your Serial No and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -27333,6 +28985,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T345" t="inlineStr">
+        <is>
+          <t>Select 'UniPin Voucher' as payment → enter your Serial No and PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -27412,6 +29069,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T346" t="inlineStr">
+        <is>
+          <t>At checkout, tap 'Apply' on GyFTR ePay Balance → enter your voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -27489,6 +29151,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T347" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -27566,6 +29233,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T348" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
@@ -27643,6 +29315,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T349" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -27722,6 +29399,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T350" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -27801,6 +29483,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T351" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -27878,6 +29565,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T352" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
@@ -27955,6 +29647,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T353" t="inlineStr">
+        <is>
+          <t>In the app, enter your code under 'Enter Voucher Code' and click Apply.</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
@@ -28032,6 +29729,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T354" t="inlineStr">
+        <is>
+          <t>Under purchase method, select 'Prepaid Cards and Codes' → enter your gift card code.</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
@@ -28109,6 +29811,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T355" t="inlineStr">
+        <is>
+          <t>Under purchase method, select 'Prepaid Cards and Codes' → enter your gift card code.</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
@@ -28184,6 +29891,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T356" t="inlineStr">
+        <is>
+          <t>At checkout, choose the 'Gift Card' option to redeem before paying.</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -28261,6 +29973,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T357" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
@@ -28340,6 +30057,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T358" t="inlineStr">
+        <is>
+          <t>At checkout, select 'Pay via e-pay/Gift Vouchers' → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -28417,6 +30139,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T359" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -28494,6 +30221,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T360" t="inlineStr">
+        <is>
+          <t>Activate via SMS to 9704200300 as instructed on the card, then show the voucher code and PIN to the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -28575,6 +30307,7 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
@@ -28652,6 +30385,11 @@
       <c r="S362" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T362" t="inlineStr">
+        <is>
+          <t>At checkout, tap 'Add' to top up your e-Pay balance → enter your voucher code and click Add.</t>
         </is>
       </c>
     </row>
@@ -28734,6 +30472,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T363" t="inlineStr">
+        <is>
+          <t>After OTP verification, your linked vouchers appear at checkout -- tap 'Redeem' to add the amount to your wallet.</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
@@ -28818,6 +30561,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T364" t="inlineStr">
+        <is>
+          <t>In the GyFTR ePay app, tap Redeem → enter amount → show the QR code to the cashier.</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
@@ -28897,6 +30645,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T365" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number with the cashier before billing.</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -28972,6 +30725,11 @@
       <c r="S366" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T366" t="inlineStr">
+        <is>
+          <t>Show voucher code to cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -29052,6 +30810,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T367" t="inlineStr">
+        <is>
+          <t>At checkout, select 'e-Pay' → verify with OTP → add your voucher to your e-Pay balance.</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -29129,6 +30892,11 @@
       <c r="S368" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T368" t="inlineStr">
+        <is>
+          <t>Share your registered mobile number or voucher code with the cashier before billing.</t>
         </is>
       </c>
     </row>
@@ -29211,6 +30979,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T369" t="inlineStr">
+        <is>
+          <t>At checkout, use the GyFTR EPAY option to redeem your voucher.</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
@@ -29291,6 +31064,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T370" t="inlineStr">
+        <is>
+          <t>Give your phone number to the cashier -- they'll check your Wow! e-Pay balance and redeem it with an OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
@@ -29371,6 +31149,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T371" t="inlineStr">
+        <is>
+          <t>Give your phone number to the cashier -- they'll check your Wow! e-Pay balance and redeem it with an OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
@@ -29451,6 +31234,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T372" t="inlineStr">
+        <is>
+          <t>Give your phone number to the cashier -- they'll check your Wow! e-Pay balance and redeem it with an OTP.</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
@@ -29526,6 +31314,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T373" t="inlineStr">
+        <is>
+          <t>At payment, tap 'Add Promo Code' → enter your code and pay Rs.1 to activate.</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
@@ -29603,6 +31396,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T374" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Vouchers' → enter your gift card details and click Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -29676,6 +31474,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T375" t="inlineStr">
+        <is>
+          <t>At payment, select 'Gift Vouchers' → enter your gift card number and press Redeem.</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -29753,6 +31556,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T376" t="inlineStr">
+        <is>
+          <t>On the plan page, tap 'Buy Plan' → enter your code under 'Apply Code' and proceed.</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -29828,6 +31636,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T377" t="inlineStr">
+        <is>
+          <t>Tap the top-left icon → 'Zepto Cash and Gift Card' → 'Add Card' → enter your 16-digit code + 6-digit PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
@@ -29903,6 +31716,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T378" t="inlineStr">
+        <is>
+          <t>Under profile → 'Credits and gift cards', tap 'Claim Gift Card' → enter your 16-digit code + PIN.</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
@@ -29980,6 +31798,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="T379" t="inlineStr">
+        <is>
+          <t>Under 'Zoom Cash', tap 'Claim a Gift Card' → choose GyFTR → enter your voucher code and click Add.</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
@@ -30057,6 +31880,11 @@
       <c r="S380" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr">
+        <is>
+          <t>At payment, select 'Add Balance to GyFTR E-Pay' and enter your voucher code.</t>
         </is>
       </c>
     </row>
@@ -30130,6 +31958,11 @@
       <c r="S381" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="T381" t="inlineStr">
+        <is>
+          <t>At checkout, choose 'Have a Promo Code' to enter your Gift Card.</t>
         </is>
       </c>
     </row>

</xml_diff>